<commit_message>
add created date as request date when sending
</commit_message>
<xml_diff>
--- a/src/main/resources/assets/template/ExportSendingTemplate.xlsx
+++ b/src/main/resources/assets/template/ExportSendingTemplate.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28730"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29029"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Backend\kvc-wh-be\target\classes\assets\template\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Project_Code\kvc-wh-be\src\main\resources\assets\template\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A5DB410-0E07-43A1-A9AC-57FD3D211125}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4BB3D50F-9BAC-45AD-9A33-15349FC9A7ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="1710" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tồn kho" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0" iterateDelta="1E-4"/>
+  <calcPr calcId="0"/>
   <extLst>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
       <loext:extCalcPr stringRefSyntax="CalcA1ExcelA1"/>
@@ -36,7 +36,7 @@
     <t>INSP DATE</t>
   </si>
   <si>
-    <t>QTY SYSTEM</t>
+    <t>REQUEST DATE</t>
   </si>
 </sst>
 </file>
@@ -390,15 +390,15 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="12.7109375" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="20.21875" style="3" customWidth="1"/>
-    <col min="2" max="2" width="25.44140625" style="5" customWidth="1"/>
-    <col min="3" max="3" width="28.5546875" customWidth="1"/>
-    <col min="4" max="4" width="27.77734375" customWidth="1"/>
+    <col min="1" max="1" width="20.28515625" style="3" customWidth="1"/>
+    <col min="2" max="2" width="25.42578125" style="5" customWidth="1"/>
+    <col min="3" max="3" width="28.5703125" customWidth="1"/>
+    <col min="4" max="4" width="20" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A1" s="2" t="s">
         <v>2</v>
       </c>
@@ -408,7 +408,7 @@
       <c r="C1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
     </row>

</xml_diff>

<commit_message>
add form code into export sending file and import sending file; update status base on form code, PO and inspection date
</commit_message>
<xml_diff>
--- a/src/main/resources/assets/template/ExportSendingTemplate.xlsx
+++ b/src/main/resources/assets/template/ExportSendingTemplate.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Project_Code\kvc-wh-be\src\main\resources\assets\template\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4BB3D50F-9BAC-45AD-9A33-15349FC9A7ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{525F1430-AD57-4100-89DA-62E6251E2042}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
   <si>
     <t>PO</t>
   </si>
@@ -37,6 +37,9 @@
   </si>
   <si>
     <t>REQUEST DATE</t>
+  </si>
+  <si>
+    <t>FORM CODE</t>
   </si>
 </sst>
 </file>
@@ -389,16 +392,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D1"/>
+  <dimension ref="A1:E1"/>
   <sheetFormatPr defaultColWidth="12.7109375" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="20.28515625" style="3" customWidth="1"/>
     <col min="2" max="2" width="25.42578125" style="5" customWidth="1"/>
     <col min="3" max="3" width="28.5703125" customWidth="1"/>
     <col min="4" max="4" width="20" customWidth="1"/>
+    <col min="5" max="5" width="16.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A1" s="2" t="s">
         <v>2</v>
       </c>
@@ -411,6 +415,9 @@
       <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
+      <c r="E1" s="2" t="s">
+        <v>4</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.74791666666666701" right="0.74791666666666701" top="0.98402777777777795" bottom="0.98402777777777795" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>